<commit_message>
refactor: reestructurar espacio de trabajo, sincronizar Markdown con Word, resolver bug de métricas undefined en el tablero y habilitar equidad por edad
</commit_message>
<xml_diff>
--- a/paper/tables/anthropic/reporte_completo_sistac.xlsx
+++ b/paper/tables/anthropic/reporte_completo_sistac.xlsx
@@ -631,7 +631,331 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Métricas de Eficiencia (H1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: Comparar el tiempo de procesamiento por candidato en segundos (Mann-Whitney U y Speedup).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>median_c0</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>median_cx</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>iqr_c0</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>iqr_cx</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>speedup</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>mannwhitney_u</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>p_value</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>h1_accepted</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>C1 (LLM puro)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>661.8</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>392.5</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>147.8x</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>C2 (LLM + RAG)</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>661.8</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>392.5</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>96.7x</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>C3 (LLM + RAG + PII)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>661.8</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>392.5</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>33.7x</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Métricas de Eficacia (H2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: Evaluar la precisión global F1-Score y AUC-ROC frente al Gold Standard (umbral F1 &gt;= 0.85).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>auc_roc</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>auc_ci</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>h2_accepted</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>C1 (LLM puro)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>0.5649999999999999</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>0.732</v>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>(0.643, 0.815)</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>C2 (LLM + RAG)</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>0.519</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>0.735</v>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>(0.651, 0.815)</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>C3 (LLM + RAG + PII)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>0.539</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>(0.639, 0.810)</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -645,14 +969,14 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Métricas de Eficiencia (H1)</t>
+          <t>Métricas de Equidad (H3)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Objetivo: Comparar el tiempo de procesamiento por candidato en segundos (Mann-Whitney U y Speedup).</t>
+          <t>Objetivo: Verificar el impacto dispar (DIR) y diferencia de paridad estadística (SPD) por género (umbral DIR &gt;= 0.80).</t>
         </is>
       </c>
     </row>
@@ -665,265 +989,57 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>median_c0</t>
+          <t>dir_gender</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>median_cx</t>
+          <t>spd_gender</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>speedup</t>
+          <t>dir_age</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>p_value</t>
+          <t>spd_age</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>h1_accepted</t>
+          <t>h3_accepted</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>C1 (LLM puro)</t>
+          <t>C2 (LLM + RAG)</t>
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>661.8</v>
+        <v>0.602</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>147.8x</t>
-        </is>
+        <v>-0.078</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>0.773</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>C2 (LLM + RAG)</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="n">
-        <v>661.8</v>
-      </c>
-      <c r="C6" s="10" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>96.7x</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>C3 (LLM + RAG + PII)</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n">
-        <v>661.8</v>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>33.7x</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Métricas de Eficacia (H2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: Evaluar la precisión global F1-Score y AUC-ROC frente al Gold Standard (umbral F1 &gt;= 0.85).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>config</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>f1</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>auc_roc</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>C1 (LLM puro)</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n">
-        <v>0.5649999999999999</v>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>0.732</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>C2 (LLM + RAG)</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="n">
-        <v>0.519</v>
-      </c>
-      <c r="C6" s="10" t="n">
-        <v>0.735</v>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>C3 (LLM + RAG + PII)</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n">
-        <v>0.539</v>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>0.729</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Métricas de Equidad (H3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: Verificar el impacto dispar (DIR) y diferencia de paridad estadística (SPD) por género (umbral DIR &gt;= 0.80).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>config</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>dir</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>spd</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>C2 (LLM + RAG)</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n">
-        <v>0.602</v>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>-0.078</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
           <t>C3 (LLM + RAG + PII)</t>
         </is>
       </c>
@@ -932,6 +1048,17 @@
       </c>
       <c r="C6" s="10" t="n">
         <v>-0.137</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>0.727</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>